<commit_message>
Complete MyAppointment, WorkSchedule and Medical test progress
</commit_message>
<xml_diff>
--- a/TestCases/Appointment_TestCase.xlsx
+++ b/TestCases/Appointment_TestCase.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DoAnNganh\SpringMediCareWeb-Selenium-Testing\TestCases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5A22C40-E7C9-4508-8735-ADD7FB3472A1}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96A7480D-F5ED-4C93-B6A2-43D11132F9E6}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="12792" windowHeight="6960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="APPOINTMENT" sheetId="6" r:id="rId1"/>
+    <sheet name="APPOINTMENT" sheetId="7" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="ACTION">#REF!</definedName>
@@ -28,6 +28,15 @@
     <t>TEST CASE</t>
   </si>
   <si>
+    <t>Pass</t>
+  </si>
+  <si>
+    <t>Fail</t>
+  </si>
+  <si>
+    <t>Pending</t>
+  </si>
+  <si>
     <t>System Name：</t>
   </si>
   <si>
@@ -38,15 +47,6 @@
   </si>
   <si>
     <t>Test requirement:</t>
-  </si>
-  <si>
-    <t>Pass</t>
-  </si>
-  <si>
-    <t>Pending</t>
-  </si>
-  <si>
-    <t>Fail</t>
   </si>
   <si>
     <t>Number of test cases:</t>
@@ -85,10 +85,10 @@
     <t>Retest Evidence</t>
   </si>
   <si>
-    <t>APPOINTMENT300 - Appointment Management</t>
+    <t>APPOINTMENT - Appointment Management</t>
   </si>
   <si>
-    <t>APPOINTMENT1 - Manage Appointment and Examination</t>
+    <t>Appointment Management and Examination</t>
   </si>
   <si>
     <t>1. Kiểm tra lịch được chuyển đến Admin</t>
@@ -97,27 +97,18 @@
     <t>TC-APPOINTMENT-001</t>
   </si>
   <si>
-    <t>Lịch hẹn bệnh nhân vừa đặt được gửi đến trang Quản lý lịch hẹn của Admin.</t>
+    <t>Kiểm tra lịch hẹn bệnh nhân vừa đặt được hiển thị đúng trên trang Quản lý lịch hẹn của Admin.</t>
   </si>
   <si>
-    <t>1: Đăng nhập bằng tài khoản bệnh nhân.
-2: Chọn bác sĩ có lịch làm việc.
-3: Chọn ngày và giờ hợp lệ, chưa có người đặt.
-4: Nhập ghi chú nhận diện TC-APPOINTMENT-001.
-5: Nhấn nút Đặt lịch.
-6: Đăng xuất và đăng nhập bằng tài khoản Admin.
-7: Mở trang Quản lý lịch hẹn.
-8: Tìm lịch có ghi chú TC-APPOINTMENT-001.</t>
+    <t>1: Đăng nhập bằng tài khoản bệnh nhân và mở trang đặt lịch của bác sĩ có lịch làm việc.
+2: Chọn ngày, giờ hợp lệ và nhập ghi chú TC-APPOINTMENT-001.
+3: Nhấn Đặt lịch và kiểm tra đặt lịch thành công.
+4: Đăng xuất và đăng nhập bằng tài khoản Admin.
+5: Mở trang Quản lý lịch hẹn và tìm lịch vừa tạo.
+6: Kiểm tra thông tin và trạng thái của lịch.</t>
   </si>
   <si>
-    <t>Bệnh nhân đặt lịch thành công.
-Admin nhìn thấy đúng lịch vừa được bệnh nhân đặt, bao gồm:
-- Đúng bệnh nhân.
-- Đúng bác sĩ.
-- Đúng ngày và giờ khám.
-- Đúng ghi chú.
-- Trạng thái Chờ xác nhận.
-- Có nút Xác nhận và Hủy.</t>
+    <t>Lịch được tạo thành công và hiển thị cho Admin với đúng bệnh nhân, bác sĩ, ngày giờ, ghi chú; trạng thái Chờ xác nhận và có nút Xác nhận, Hủy.</t>
   </si>
   <si>
     <t xml:space="preserve">TCAppointment1_1, TCAppointment1_2, TCAppointment1_3 </t>
@@ -132,24 +123,17 @@
     <t>TC-APPOINTMENT-002</t>
   </si>
   <si>
-    <t>Admin xác nhận thành công lịch hẹn đang chờ xác nhận.</t>
+    <t>Kiểm tra Admin xác nhận thành công lịch hẹn đang ở trạng thái Chờ xác nhận.</t>
   </si>
   <si>
-    <t>1: Đăng nhập bằng tài khoản Admin.
-2: Mở trang Quản lý lịch hẹn.
-3: Tìm lịch TC-APPOINTMENT-002.
-4: Kiểm tra lịch đang ở trạng thái Chờ xác nhận.
-5: Nhấn nút Xác nhận.
-6: Đồng ý trên hộp thoại xác nhận.
-7: Tải lại trang.
-8: Kiểm tra trạng thái và các nút thao tác.</t>
+    <t>1: Đăng nhập Admin và mở trang Quản lý lịch hẹn.
+2: Tìm lịch TC-APPOINTMENT-002 đang ở trạng thái Chờ xác nhận.
+3: Nhấn Xác nhận và đồng ý trên hộp thoại xác nhận.
+4: Kiểm tra thông báo xác nhận thành công.
+5: Kiểm tra trạng thái và thông tin lịch sau khi xác nhận.</t>
   </si>
   <si>
-    <t>Hệ thống hiển thị thông báo xác nhận thành công.
-Trạng thái lịch chuyển từ Chờ xác nhận sang Đã xác nhận.
-Nút Xác nhận và Hủy không còn hiển thị.
-Thông tin bệnh nhân, bác sĩ, thời gian và ghi chú không bị thay đổi.
-Hệ thống không tạo thêm lịch hẹn mới.</t>
+    <t>Trạng thái chuyển sang Đã xác nhận; nút Xác nhận, Hủy không còn hiển thị; thông tin lịch không thay đổi.</t>
   </si>
   <si>
     <t>TCAppointment2_1, TCAppointment2_2</t>
@@ -161,23 +145,17 @@
     <t>TC-APPOINTMENT-003</t>
   </si>
   <si>
-    <t>Admin hủy thành công lịch hẹn đang chờ xác nhận.</t>
+    <t>Kiểm tra Admin hủy thành công lịch hẹn đang chờ xác nhận.</t>
   </si>
   <si>
-    <t>1: Đăng nhập bằng tài khoản Admin.
-2: Mở trang Quản lý lịch hẹn.
-3: Tìm lịch TC-APPOINTMENT-003.
-4: Kiểm tra lịch đang ở trạng thái Chờ xác nhận.
-5: Nhấn nút Hủy.
-6: Đồng ý trên hộp thoại xác nhận.
-7: Tải lại trang.
-8: Kiểm tra trạng thái và các nút thao tác.</t>
+    <t>1: Đăng nhập Admin và mở trang Quản lý lịch hẹn.
+2: Tìm lịch TC-APPOINTMENT-003 đang ở trạng thái Chờ xác nhận.
+3: Nhấn Hủy và đồng ý trên hộp thoại xác nhận.
+4: Kiểm tra thông báo hủy lịch thành công.
+5: Kiểm tra trạng thái và thông tin lịch sau khi hủy.</t>
   </si>
   <si>
-    <t>Hệ thống hiển thị thông báo hủy lịch thành công.
-Trạng thái lịch chuyển từ Chờ xác nhận sang Đã hủy.
-Nút Xác nhận và Hủy không còn hiển thị.
-Thông tin bệnh nhân, bác sĩ, thời gian và ghi chú không bị thay đổi.</t>
+    <t>Trạng thái chuyển sang Đã hủy; nút Xác nhận, Hủy không còn hiển thị; thông tin lịch không thay đổi.</t>
   </si>
   <si>
     <t>TCAppointment3_1, TCAppointment3_2, TCAppointment3_3</t>
@@ -192,23 +170,17 @@
     <t>TC-APPOINTMENT-004</t>
   </si>
   <si>
-    <t>Bác sĩ chỉ được xem hồ sơ bệnh nhân khi lịch chưa được Admin xác nhận.</t>
+    <t>Kiểm tra quyền xem hồ sơ bệnh nhân của bác sĩ khi lịch đang chờ xác nhận.</t>
   </si>
   <si>
     <t>1: Đăng nhập bằng đúng tài khoản bác sĩ của lịch.
-2: Mở trang Lịch hẹn bệnh nhân.
-3: Tìm lịch TC-APPOINTMENT-004.
-4: Kiểm tra trạng thái của lịch.
-5: Kiểm tra các nút thao tác.
-6: Nhấn nút Xem hồ sơ.
-7: Kiểm tra thông tin hồ sơ bệnh nhân.</t>
+2: Mở trang Lịch hẹn bệnh nhân và tìm lịch TC-APPOINTMENT-004.
+3: Kiểm tra trạng thái và các nút thao tác của lịch.
+4: Nhấn Xem hồ sơ.
+5: Kiểm tra hồ sơ/lịch sử khám của bệnh nhân.</t>
   </si>
   <si>
-    <t>Bác sĩ nhìn thấy lịch hẹn thuộc mình.
-Lịch hiển thị trạng thái Chờ xác nhận.
-Bác sĩ được phép xem hồ sơ hoặc lịch sử khám của bệnh nhân.
-Không hiển thị nút Khám bệnh.
-Bác sĩ không thể tạo hồ sơ bệnh án mới cho lịch này.</t>
+    <t>Lịch ở trạng thái Chờ xác nhận; bác sĩ được xem hồ sơ/lịch sử khám nhưng không có nút Khám bệnh và không thể tạo hồ sơ bệnh án mới.</t>
   </si>
   <si>
     <t>TCAppointment4</t>
@@ -220,22 +192,17 @@
     <t>TC-APPOINTMENT-005</t>
   </si>
   <si>
-    <t>Bác sĩ truy cập trực tiếp trang khám của lịch chưa được xác nhận.</t>
+    <t>Kiểm tra bác sĩ không thể truy cập trực tiếp trang khám của lịch chưa được Admin xác nhận.</t>
   </si>
   <si>
-    <t>1: Đăng nhập bằng đúng tài khoản bác sĩ của lịch.
-2: Lấy appointmentId của lịch TC-APPOINTMENT-005.
-3: Nhập trực tiếp URL trang khám có appointmentId đó.
-4: Kiểm tra nội dung trang được hiển thị.
-5: Thử nhập thông tin khám nếu form vẫn xuất hiện.
-6: Thử nhấn nút Lưu hồ sơ.
-7: Kiểm tra trạng thái lịch và dữ liệu hồ sơ.</t>
+    <t>1: Đăng nhập bằng đúng tài khoản bác sĩ của lịch TC-APPOINTMENT-005.
+2: Truy cập trực tiếp URL trang khám bằng appointmentId của lịch.
+3: Kiểm tra phản hồi của hệ thống.
+4: Kiểm tra không thể thực hiện và lưu thông tin khám.
+5: Kiểm tra trạng thái lịch và dữ liệu hồ sơ.</t>
   </si>
   <si>
-    <t>Hệ thống không cho phép bác sĩ thực hiện khám bệnh.
-Trang khám bị chặn, chuyển hướng hoặc hiển thị thông báo lịch chưa được xác nhận.
-Không tạo hồ sơ bệnh án.
-Trạng thái lịch vẫn là Chờ xác nhận.</t>
+    <t>Trang khám bị chặn, chuyển hướng hoặc thông báo lịch chưa được xác nhận; không tạo hồ sơ bệnh án; lịch vẫn ở trạng thái Chờ xác nhận.</t>
   </si>
   <si>
     <t>TCAppointment5_1, TCAppointment5_2</t>
@@ -250,24 +217,17 @@
     <t>TC-APPOINTMENT-006</t>
   </si>
   <si>
-    <t>Đúng bác sĩ được mở chức năng khám bệnh khi lịch đã được Admin xác nhận.</t>
+    <t>Kiểm tra đúng bác sĩ được phép khám bệnh khi lịch đã được xác nhận.</t>
   </si>
   <si>
     <t>1: Đăng nhập bằng đúng tài khoản bác sĩ của lịch.
-2: Mở trang Lịch hẹn bệnh nhân.
-3: Tìm lịch TC-APPOINTMENT-006.
-4: Kiểm tra trạng thái của lịch.
-5: Kiểm tra nút Khám bệnh.
-6: Nhấn nút Khám bệnh.
-7: Kiểm tra thông tin bệnh nhân và lịch hẹn.
-8: Kiểm tra form nhập kết quả khám.</t>
+2: Mở trang Lịch hẹn bệnh nhân và tìm lịch TC-APPOINTMENT-006.
+3: Kiểm tra lịch ở trạng thái Đã xác nhận và có nút Khám bệnh.
+4: Nhấn Khám bệnh.
+5: Kiểm tra thông tin bệnh nhân và form khám được hiển thị.</t>
   </si>
   <si>
-    <t>Lịch hiển thị trạng thái Đã xác nhận.
-Hệ thống hiển thị nút Khám bệnh.
-Khi nhấn Khám bệnh, hệ thống mở đúng lịch và đúng bệnh nhân.
-Trang khám hiển thị form nhập chẩn đoán và hướng điều trị.
-Trạng thái lịch vẫn là Đã xác nhận khi chưa lưu hồ sơ.</t>
+    <t>Trang khám mở đúng lịch và bệnh nhân; hiển thị form nhập chẩn đoán, hướng điều trị; lịch vẫn Đã xác nhận khi chưa lưu hồ sơ.</t>
   </si>
   <si>
     <t>TCAppointment6_1, TCAppointment6_2</t>
@@ -279,23 +239,17 @@
     <t>TC-APPOINTMENT-007</t>
   </si>
   <si>
-    <t>Bác sĩ không được khám lịch hẹn đã xác nhận nhưng không thuộc mình.</t>
+    <t>Kiểm tra bác sĩ khác không thể khám lịch hẹn không thuộc mình.</t>
   </si>
   <si>
-    <t>1: Đăng nhập bằng một bác sĩ khác với bác sĩ của lịch.
-2: Mở trang Lịch hẹn bệnh nhân.
-3: Tìm lịch TC-APPOINTMENT-007.
-4: Kiểm tra lịch có xuất hiện hay không.
-5: Nhập trực tiếp URL trang khám của lịch đó.
-6: Quan sát phản hồi của hệ thống.
-7: Kiểm tra trạng thái lịch và dữ liệu hồ sơ.</t>
+    <t>1: Đăng nhập bằng tài khoản bác sĩ khác với bác sĩ của lịch TC-APPOINTMENT-007.
+2: Mở trang Lịch hẹn bệnh nhân và kiểm tra lịch không xuất hiện.
+3: Truy cập trực tiếp URL trang khám bằng appointmentId của lịch.
+4: Kiểm tra phản hồi của hệ thống.
+5: Kiểm tra trạng thái lịch và dữ liệu hồ sơ.</t>
   </si>
   <si>
-    <t>Lịch không xuất hiện trong danh sách của bác sĩ khác.
-Bác sĩ khác không được mở trang khám của lịch.
-Hệ thống hiển thị thông báo không có quyền hoặc chuyển hướng.
-Không tạo hồ sơ bệnh án.
-Trạng thái lịch không thay đổi.</t>
+    <t>Lịch không xuất hiện trong danh sách; truy cập trực tiếp bị chặn/chuyển hướng hoặc báo không có quyền; không tạo hồ sơ bệnh án và trạng thái lịch không thay đổi.</t>
   </si>
   <si>
     <t>TCAppointment7_1, TCAppointment7_2</t>
@@ -310,23 +264,17 @@
     <t>TC-APPOINTMENT-008</t>
   </si>
   <si>
-    <t>Bác sĩ không được khám bệnh đối với lịch đã bị Admin hủy.</t>
+    <t>Kiểm tra bác sĩ không thể khám bệnh đối với lịch đã bị hủy.</t>
   </si>
   <si>
     <t>1: Đăng nhập bằng đúng tài khoản bác sĩ của lịch.
-2: Mở trang Lịch hẹn bệnh nhân.
-3: Tìm lịch TC-APPOINTMENT-008.
-4: Kiểm tra trạng thái của lịch.
-5: Kiểm tra các nút thao tác.
-6: Nhập trực tiếp URL trang khám của lịch.
-7: Kiểm tra phản hồi của hệ thống.</t>
+2: Mở trang Lịch hẹn bệnh nhân và tìm lịch TC-APPOINTMENT-008.
+3: Kiểm tra lịch ở trạng thái Đã hủy và không có nút Khám bệnh.
+4: Truy cập trực tiếp URL trang khám bằng appointmentId của lịch.
+5: Kiểm tra phản hồi và dữ liệu của lịch.</t>
   </si>
   <si>
-    <t>Lịch hiển thị trạng thái Đã hủy.
-Không hiển thị nút Khám bệnh.
-Truy cập trực tiếp trang khám bị chặn hoặc chuyển hướng.
-Không tạo hồ sơ bệnh án.
-Trạng thái lịch vẫn là Đã hủy.</t>
+    <t>Không có nút Khám bệnh; truy cập trực tiếp trang khám bị chặn/chuyển hướng; không tạo hồ sơ bệnh án; trạng thái vẫn Đã hủy.</t>
   </si>
   <si>
     <t>TCAppointment8_1, TCAppointment8_2</t>
@@ -344,24 +292,18 @@
     <t>TC-APPOINTMENT-009</t>
   </si>
   <si>
-    <t>Bác sĩ lưu hồ sơ bệnh án và hoàn thành lịch đã xác nhận.</t>
+    <t>Kiểm tra bác sĩ lưu hồ sơ bệnh án và hoàn thành lịch hẹn đã xác nhận.</t>
   </si>
   <si>
-    <t>1: Đăng nhập bằng đúng tài khoản bác sĩ của lịch.
-2: Mở trang Lịch hẹn bệnh nhân.
-3: Tìm lịch TC-APPOINTMENT-009.
-4: Nhấn nút Khám bệnh.
-5: Nhập chẩn đoán và hướng điều trị hợp lệ.
-6: Nhấn nút Lưu hồ sơ.
-7: Quay lại danh sách lịch hẹn.
-8: Kiểm tra trạng thái và hồ sơ vừa tạo.</t>
+    <t>1: Đăng nhập bằng đúng tài khoản bác sĩ và mở lịch TC-APPOINTMENT-009 đã được xác nhận.
+2: Nhấn Khám bệnh.
+3: Nhập chẩn đoán và hướng điều trị hợp lệ.
+4: Nhấn Lưu hồ sơ và kiểm tra lưu thành công.
+5: Quay lại danh sách lịch hẹn và kiểm tra trạng thái.
+6: Mở lại hồ sơ và kiểm tra thông tin vừa lưu.</t>
   </si>
   <si>
-    <t>Hệ thống lưu hồ sơ bệnh án thành công.
-Hồ sơ được gắn đúng với bệnh nhân, bác sĩ và appointmentId.
-Trạng thái lịch chuyển từ Đã xác nhận sang Đã hoàn thành.
-Không còn hiển thị nút Khám bệnh.
-Bác sĩ có thể mở và xem lại hồ sơ đã tạo.</t>
+    <t>Hồ sơ bệnh án được lưu đúng bệnh nhân, bác sĩ và lịch hẹn; trạng thái chuyển sang Đã hoàn thành; không còn nút Khám bệnh và có thể xem lại hồ sơ.</t>
   </si>
   <si>
     <t>TCAppointment9_1, TCAppointment9_2, TCAppointment9_3</t>
@@ -642,33 +584,33 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -895,7 +837,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -918,9 +860,9 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
@@ -947,9 +889,9 @@
     </row>
     <row r="2" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
@@ -976,13 +918,13 @@
     </row>
     <row r="3" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>1</v>
+        <v>4</v>
       </c>
-      <c r="B3" s="32" t="s">
-        <v>2</v>
+      <c r="B3" s="28" t="s">
+        <v>5</v>
       </c>
-      <c r="C3" s="25"/>
-      <c r="D3" s="27"/>
+      <c r="C3" s="29"/>
+      <c r="D3" s="30"/>
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
@@ -1009,13 +951,13 @@
     </row>
     <row r="4" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
-      <c r="B4" s="33" t="s">
+      <c r="B4" s="31" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="25"/>
-      <c r="D4" s="27"/>
+      <c r="C4" s="29"/>
+      <c r="D4" s="30"/>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
@@ -1042,13 +984,13 @@
     </row>
     <row r="5" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
-      <c r="B5" s="32" t="s">
+      <c r="B5" s="28" t="s">
         <v>21</v>
       </c>
-      <c r="C5" s="25"/>
-      <c r="D5" s="27"/>
+      <c r="C5" s="29"/>
+      <c r="D5" s="30"/>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
@@ -1075,13 +1017,13 @@
     </row>
     <row r="6" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="B6" s="6">
         <v>5</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D6" s="8">
         <v>0</v>
@@ -1112,7 +1054,7 @@
     </row>
     <row r="7" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="B7" s="6">
         <v>4</v>
@@ -1177,21 +1119,21 @@
       <c r="AA8" s="3"/>
     </row>
     <row r="9" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A9" s="34" t="s">
+      <c r="A9" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="35" t="s">
+      <c r="B9" s="34" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="34" t="s">
+      <c r="C9" s="32" t="s">
         <v>11</v>
       </c>
-      <c r="D9" s="36" t="s">
+      <c r="D9" s="35" t="s">
         <v>12</v>
       </c>
-      <c r="E9" s="31"/>
-      <c r="F9" s="31"/>
-      <c r="G9" s="34" t="s">
+      <c r="E9" s="25"/>
+      <c r="F9" s="25"/>
+      <c r="G9" s="32" t="s">
         <v>13</v>
       </c>
       <c r="H9" s="37" t="s">
@@ -1228,19 +1170,19 @@
       <c r="AA9" s="3"/>
     </row>
     <row r="10" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A10" s="26"/>
-      <c r="B10" s="26"/>
-      <c r="C10" s="26"/>
-      <c r="D10" s="28"/>
-      <c r="E10" s="29"/>
-      <c r="F10" s="29"/>
-      <c r="G10" s="26"/>
-      <c r="H10" s="26"/>
-      <c r="I10" s="26"/>
-      <c r="J10" s="26"/>
-      <c r="K10" s="26"/>
-      <c r="L10" s="26"/>
-      <c r="M10" s="26"/>
+      <c r="A10" s="33"/>
+      <c r="B10" s="33"/>
+      <c r="C10" s="33"/>
+      <c r="D10" s="36"/>
+      <c r="E10" s="27"/>
+      <c r="F10" s="27"/>
+      <c r="G10" s="33"/>
+      <c r="H10" s="33"/>
+      <c r="I10" s="33"/>
+      <c r="J10" s="33"/>
+      <c r="K10" s="33"/>
+      <c r="L10" s="33"/>
+      <c r="M10" s="33"/>
       <c r="N10" s="3"/>
       <c r="O10" s="3"/>
       <c r="P10" s="3"/>
@@ -1263,13 +1205,13 @@
       <c r="D11" s="11"/>
       <c r="E11" s="11"/>
       <c r="F11" s="38"/>
-      <c r="G11" s="25"/>
-      <c r="H11" s="25"/>
-      <c r="I11" s="25"/>
-      <c r="J11" s="25"/>
-      <c r="K11" s="25"/>
-      <c r="L11" s="25"/>
-      <c r="M11" s="25"/>
+      <c r="G11" s="29"/>
+      <c r="H11" s="29"/>
+      <c r="I11" s="29"/>
+      <c r="J11" s="29"/>
+      <c r="K11" s="29"/>
+      <c r="L11" s="29"/>
+      <c r="M11" s="29"/>
       <c r="N11" s="3"/>
       <c r="O11" s="3"/>
       <c r="P11" s="3"/>
@@ -1289,18 +1231,18 @@
       <c r="A12" s="39" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="25"/>
-      <c r="C12" s="25"/>
-      <c r="D12" s="25"/>
-      <c r="E12" s="25"/>
-      <c r="F12" s="25"/>
-      <c r="G12" s="25"/>
-      <c r="H12" s="25"/>
-      <c r="I12" s="25"/>
-      <c r="J12" s="25"/>
-      <c r="K12" s="25"/>
-      <c r="L12" s="25"/>
-      <c r="M12" s="27"/>
+      <c r="B12" s="29"/>
+      <c r="C12" s="29"/>
+      <c r="D12" s="29"/>
+      <c r="E12" s="29"/>
+      <c r="F12" s="29"/>
+      <c r="G12" s="29"/>
+      <c r="H12" s="29"/>
+      <c r="I12" s="29"/>
+      <c r="J12" s="29"/>
+      <c r="K12" s="29"/>
+      <c r="L12" s="29"/>
+      <c r="M12" s="30"/>
       <c r="N12" s="3"/>
       <c r="O12" s="3"/>
       <c r="P12" s="3"/>
@@ -1316,7 +1258,7 @@
       <c r="Z12" s="3"/>
       <c r="AA12" s="3"/>
     </row>
-    <row r="13" spans="1:27" ht="122.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:27" ht="135.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
         <v>23</v>
       </c>
@@ -1329,8 +1271,8 @@
       <c r="D13" s="40" t="s">
         <v>26</v>
       </c>
-      <c r="E13" s="25"/>
-      <c r="F13" s="25"/>
+      <c r="E13" s="29"/>
+      <c r="F13" s="29"/>
       <c r="G13" s="17" t="s">
         <v>27</v>
       </c>
@@ -1338,7 +1280,7 @@
         <v>46232</v>
       </c>
       <c r="I13" s="14" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J13" s="16" t="s">
         <v>28</v>
@@ -1365,18 +1307,18 @@
       <c r="A14" s="39" t="s">
         <v>29</v>
       </c>
-      <c r="B14" s="25"/>
-      <c r="C14" s="25"/>
-      <c r="D14" s="25"/>
-      <c r="E14" s="25"/>
-      <c r="F14" s="25"/>
-      <c r="G14" s="25"/>
-      <c r="H14" s="25"/>
-      <c r="I14" s="25"/>
-      <c r="J14" s="25"/>
-      <c r="K14" s="25"/>
-      <c r="L14" s="25"/>
-      <c r="M14" s="27"/>
+      <c r="B14" s="29"/>
+      <c r="C14" s="29"/>
+      <c r="D14" s="29"/>
+      <c r="E14" s="29"/>
+      <c r="F14" s="29"/>
+      <c r="G14" s="29"/>
+      <c r="H14" s="29"/>
+      <c r="I14" s="29"/>
+      <c r="J14" s="29"/>
+      <c r="K14" s="29"/>
+      <c r="L14" s="29"/>
+      <c r="M14" s="30"/>
       <c r="N14" s="3"/>
       <c r="O14" s="3"/>
       <c r="P14" s="3"/>
@@ -1405,8 +1347,8 @@
       <c r="D15" s="40" t="s">
         <v>33</v>
       </c>
-      <c r="E15" s="25"/>
-      <c r="F15" s="25"/>
+      <c r="E15" s="29"/>
+      <c r="F15" s="29"/>
       <c r="G15" s="17" t="s">
         <v>34</v>
       </c>
@@ -1414,7 +1356,7 @@
         <v>46232</v>
       </c>
       <c r="I15" s="14" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J15" s="16" t="s">
         <v>35</v>
@@ -1450,8 +1392,8 @@
       <c r="D16" s="40" t="s">
         <v>39</v>
       </c>
-      <c r="E16" s="25"/>
-      <c r="F16" s="25"/>
+      <c r="E16" s="29"/>
+      <c r="F16" s="29"/>
       <c r="G16" s="17" t="s">
         <v>40</v>
       </c>
@@ -1459,7 +1401,7 @@
         <v>46232</v>
       </c>
       <c r="I16" s="14" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J16" s="16" t="s">
         <v>41</v>
@@ -1486,18 +1428,18 @@
       <c r="A17" s="39" t="s">
         <v>42</v>
       </c>
-      <c r="B17" s="25"/>
-      <c r="C17" s="25"/>
-      <c r="D17" s="25"/>
-      <c r="E17" s="25"/>
-      <c r="F17" s="25"/>
-      <c r="G17" s="25"/>
-      <c r="H17" s="25"/>
-      <c r="I17" s="25"/>
-      <c r="J17" s="25"/>
-      <c r="K17" s="25"/>
-      <c r="L17" s="25"/>
-      <c r="M17" s="27"/>
+      <c r="B17" s="29"/>
+      <c r="C17" s="29"/>
+      <c r="D17" s="29"/>
+      <c r="E17" s="29"/>
+      <c r="F17" s="29"/>
+      <c r="G17" s="29"/>
+      <c r="H17" s="29"/>
+      <c r="I17" s="29"/>
+      <c r="J17" s="29"/>
+      <c r="K17" s="29"/>
+      <c r="L17" s="29"/>
+      <c r="M17" s="30"/>
       <c r="N17" s="3"/>
       <c r="O17" s="3"/>
       <c r="P17" s="3"/>
@@ -1526,8 +1468,8 @@
       <c r="D18" s="40" t="s">
         <v>46</v>
       </c>
-      <c r="E18" s="25"/>
-      <c r="F18" s="25"/>
+      <c r="E18" s="29"/>
+      <c r="F18" s="29"/>
       <c r="G18" s="17" t="s">
         <v>47</v>
       </c>
@@ -1535,7 +1477,7 @@
         <v>46232</v>
       </c>
       <c r="I18" s="14" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="J18" s="16" t="s">
         <v>48</v>
@@ -1571,8 +1513,8 @@
       <c r="D19" s="40" t="s">
         <v>52</v>
       </c>
-      <c r="E19" s="25"/>
-      <c r="F19" s="25"/>
+      <c r="E19" s="29"/>
+      <c r="F19" s="29"/>
       <c r="G19" s="17" t="s">
         <v>53</v>
       </c>
@@ -1580,7 +1522,7 @@
         <v>46232</v>
       </c>
       <c r="I19" s="14" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="J19" s="16" t="s">
         <v>54</v>
@@ -1589,7 +1531,7 @@
         <v>46233</v>
       </c>
       <c r="L19" s="14" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="M19" s="21" t="s">
         <v>55</v>
@@ -1622,8 +1564,8 @@
       <c r="D20" s="40" t="s">
         <v>59</v>
       </c>
-      <c r="E20" s="25"/>
-      <c r="F20" s="25"/>
+      <c r="E20" s="29"/>
+      <c r="F20" s="29"/>
       <c r="G20" s="17" t="s">
         <v>60</v>
       </c>
@@ -1631,7 +1573,7 @@
         <v>46232</v>
       </c>
       <c r="I20" s="14" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J20" s="16" t="s">
         <v>61</v>
@@ -1667,8 +1609,8 @@
       <c r="D21" s="40" t="s">
         <v>65</v>
       </c>
-      <c r="E21" s="25"/>
-      <c r="F21" s="25"/>
+      <c r="E21" s="29"/>
+      <c r="F21" s="29"/>
       <c r="G21" s="17" t="s">
         <v>66</v>
       </c>
@@ -1676,7 +1618,7 @@
         <v>46232</v>
       </c>
       <c r="I21" s="14" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="J21" s="16" t="s">
         <v>67</v>
@@ -1685,7 +1627,7 @@
         <v>46233</v>
       </c>
       <c r="L21" s="14" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="M21" s="21" t="s">
         <v>68</v>
@@ -1718,8 +1660,8 @@
       <c r="D22" s="40" t="s">
         <v>72</v>
       </c>
-      <c r="E22" s="25"/>
-      <c r="F22" s="25"/>
+      <c r="E22" s="29"/>
+      <c r="F22" s="29"/>
       <c r="G22" s="17" t="s">
         <v>73</v>
       </c>
@@ -1727,7 +1669,7 @@
         <v>46232</v>
       </c>
       <c r="I22" s="14" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="J22" s="16" t="s">
         <v>74</v>
@@ -1736,7 +1678,7 @@
         <v>46233</v>
       </c>
       <c r="L22" s="14" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="M22" s="21" t="s">
         <v>75</v>
@@ -1746,18 +1688,18 @@
       <c r="A23" s="39" t="s">
         <v>76</v>
       </c>
-      <c r="B23" s="25"/>
-      <c r="C23" s="25"/>
-      <c r="D23" s="25"/>
-      <c r="E23" s="25"/>
-      <c r="F23" s="25"/>
-      <c r="G23" s="25"/>
-      <c r="H23" s="25"/>
-      <c r="I23" s="25"/>
-      <c r="J23" s="25"/>
-      <c r="K23" s="25"/>
-      <c r="L23" s="25"/>
-      <c r="M23" s="27"/>
+      <c r="B23" s="29"/>
+      <c r="C23" s="29"/>
+      <c r="D23" s="29"/>
+      <c r="E23" s="29"/>
+      <c r="F23" s="29"/>
+      <c r="G23" s="29"/>
+      <c r="H23" s="29"/>
+      <c r="I23" s="29"/>
+      <c r="J23" s="29"/>
+      <c r="K23" s="29"/>
+      <c r="L23" s="29"/>
+      <c r="M23" s="30"/>
       <c r="N23" s="3"/>
       <c r="O23" s="3"/>
       <c r="P23" s="3"/>
@@ -1786,8 +1728,8 @@
       <c r="D24" s="40" t="s">
         <v>80</v>
       </c>
-      <c r="E24" s="25"/>
-      <c r="F24" s="25"/>
+      <c r="E24" s="29"/>
+      <c r="F24" s="29"/>
       <c r="G24" s="17" t="s">
         <v>81</v>
       </c>
@@ -1795,14 +1737,14 @@
         <v>46232</v>
       </c>
       <c r="I24" s="14" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J24" s="16" t="s">
         <v>82</v>
       </c>
       <c r="K24" s="18"/>
       <c r="L24" s="14"/>
-      <c r="M24" s="23"/>
+      <c r="M24" s="22"/>
     </row>
     <row r="25" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A25" s="3"/>
@@ -1893,7 +1835,7 @@
     </row>
     <row r="28" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A28" s="3"/>
-      <c r="B28" s="22"/>
+      <c r="B28" s="23"/>
       <c r="C28" s="3"/>
       <c r="D28" s="3"/>
       <c r="E28" s="3"/>
@@ -2507,7 +2449,7 @@
       <c r="D49" s="3"/>
       <c r="E49" s="3"/>
       <c r="F49" s="3"/>
-      <c r="G49" s="22"/>
+      <c r="G49" s="23"/>
       <c r="H49" s="3"/>
       <c r="I49" s="3"/>
       <c r="J49" s="3"/>
@@ -30170,18 +30112,18 @@
     <mergeCell ref="D9:F10"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="G13" r:id="rId1" xr:uid="{00000000-0004-0000-0500-000000000000}"/>
-    <hyperlink ref="G15" r:id="rId2" xr:uid="{00000000-0004-0000-0500-000001000000}"/>
-    <hyperlink ref="G16" r:id="rId3" xr:uid="{00000000-0004-0000-0500-000002000000}"/>
-    <hyperlink ref="G18" r:id="rId4" xr:uid="{00000000-0004-0000-0500-000003000000}"/>
-    <hyperlink ref="G19" r:id="rId5" xr:uid="{00000000-0004-0000-0500-000004000000}"/>
-    <hyperlink ref="M19" r:id="rId6" xr:uid="{00000000-0004-0000-0500-000005000000}"/>
-    <hyperlink ref="G20" r:id="rId7" xr:uid="{00000000-0004-0000-0500-000006000000}"/>
-    <hyperlink ref="G21" r:id="rId8" xr:uid="{00000000-0004-0000-0500-000007000000}"/>
-    <hyperlink ref="M21" r:id="rId9" xr:uid="{00000000-0004-0000-0500-000008000000}"/>
-    <hyperlink ref="G22" r:id="rId10" xr:uid="{00000000-0004-0000-0500-000009000000}"/>
-    <hyperlink ref="M22" r:id="rId11" xr:uid="{00000000-0004-0000-0500-00000A000000}"/>
-    <hyperlink ref="G24" r:id="rId12" xr:uid="{00000000-0004-0000-0500-00000B000000}"/>
+    <hyperlink ref="G13" r:id="rId1" xr:uid="{00000000-0004-0000-0600-000000000000}"/>
+    <hyperlink ref="G15" r:id="rId2" xr:uid="{00000000-0004-0000-0600-000001000000}"/>
+    <hyperlink ref="G16" r:id="rId3" xr:uid="{00000000-0004-0000-0600-000002000000}"/>
+    <hyperlink ref="G18" r:id="rId4" xr:uid="{00000000-0004-0000-0600-000003000000}"/>
+    <hyperlink ref="G19" r:id="rId5" xr:uid="{00000000-0004-0000-0600-000004000000}"/>
+    <hyperlink ref="M19" r:id="rId6" xr:uid="{00000000-0004-0000-0600-000005000000}"/>
+    <hyperlink ref="G20" r:id="rId7" xr:uid="{00000000-0004-0000-0600-000006000000}"/>
+    <hyperlink ref="G21" r:id="rId8" xr:uid="{00000000-0004-0000-0600-000007000000}"/>
+    <hyperlink ref="M21" r:id="rId9" xr:uid="{00000000-0004-0000-0600-000008000000}"/>
+    <hyperlink ref="G22" r:id="rId10" xr:uid="{00000000-0004-0000-0600-000009000000}"/>
+    <hyperlink ref="M22" r:id="rId11" xr:uid="{00000000-0004-0000-0600-00000A000000}"/>
+    <hyperlink ref="G24" r:id="rId12" xr:uid="{00000000-0004-0000-0600-00000B000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>